<commit_message>
Sales products: their own catalogue lists
Categories, subcategories, attributes and tags now belong to a catalogue
(dry-hire or sales). Sales starts from its current categories, each with a
General subcategory, and tags Featured/New/Promotion. Sales form and list use
the same fields as dry-hire; import checks the sales lists (any language);
Settings > Product categories has a Dry-hire / Sales switch. Migration keeps the
old sales category in legacy_category and can be undone.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ScvRd7o1AxyUAF29FPAkVB
</commit_message>
<xml_diff>
--- a/resources/templates/CLUK_Import_Templates.xlsx
+++ b/resources/templates/CLUK_Import_Templates.xlsx
@@ -174,7 +174,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -346,6 +346,7 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -891,7 +892,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="29" t="inlineStr">
         <is>
@@ -12329,7 +12329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:X501"/>
+  <dimension ref="A1:AA501"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="29" min="1" max="2"/>
@@ -12354,6 +12354,9 @@
     <col width="14" customWidth="1" style="29" min="21" max="21"/>
     <col width="11" customWidth="1" style="29" min="22" max="22"/>
     <col width="13" customWidth="1" style="29" min="23" max="24"/>
+    <col width="18" customWidth="1" style="30" min="25" max="25"/>
+    <col width="18" customWidth="1" style="30" min="26" max="26"/>
+    <col width="18" customWidth="1" style="30" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1" s="30">
@@ -12475,6 +12478,21 @@
       <c r="X1" s="47" t="inlineStr">
         <is>
           <t>Margin at list price (calculated)</t>
+        </is>
+      </c>
+      <c r="Y1" s="35" t="inlineStr">
+        <is>
+          <t>Sub-Category</t>
+        </is>
+      </c>
+      <c r="Z1" s="35" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="AA1" s="35" t="inlineStr">
+        <is>
+          <t>Search words</t>
         </is>
       </c>
     </row>
@@ -32510,7 +32528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="30" min="1" max="1"/>
@@ -33619,7 +33637,6 @@
       </c>
       <c r="D58" s="29" t="inlineStr"/>
     </row>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="58" t="inlineStr">
         <is>
@@ -33704,7 +33721,6 @@
         </is>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" s="58" t="inlineStr">
         <is>
@@ -33717,11 +33733,118 @@
         </is>
       </c>
     </row>
-    <row r="69"/>
     <row r="70">
       <c r="A70" s="29" t="inlineStr">
         <is>
           <t>Names in Dutch, French or Spanish and the codes are accepted too. Unknown values stop that row with a clear message. The lists are managed in Settings › Product categories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="59" t="inlineStr">
+        <is>
+          <t>Sales products: categories</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Sub-Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Connectors</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Rigging</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Consumables</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Cases</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>General</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sales catalogue: brands list, manufacturer code, supplier article number
- Settings › Product categories › Brands: own / we distribute / other, with
  logo, website, text per language and a web address (old ones keep working).
  Merge two spellings; a brand in use can't be deleted.
- Typing a brand on a product uses the list's spelling or adds it.
- Manufacturer code on each sales product (our S-number stays the main number).
- Supplier's own article number editable per supplier; price requests,
  purchase orders and their PDFs show supplier no., manufacturer code and ours.
- Search on manufacturer code (with or without dashes), EAN and supplier
  article number; brand filter in the item list; import column "Manufacturer code".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ScvRd7o1AxyUAF29FPAkVB
</commit_message>
<xml_diff>
--- a/resources/templates/CLUK_Import_Templates.xlsx
+++ b/resources/templates/CLUK_Import_Templates.xlsx
@@ -12329,7 +12329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AA501"/>
+  <dimension ref="A1:AB501"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="29" min="1" max="2"/>
@@ -12357,6 +12357,7 @@
     <col width="18" customWidth="1" style="30" min="25" max="25"/>
     <col width="18" customWidth="1" style="30" min="26" max="26"/>
     <col width="18" customWidth="1" style="30" min="27" max="27"/>
+    <col width="22" customWidth="1" style="30" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1" s="30">
@@ -12493,6 +12494,11 @@
       <c r="AA1" s="35" t="inlineStr">
         <is>
           <t>Search words</t>
+        </is>
+      </c>
+      <c r="AB1" s="35" t="inlineStr">
+        <is>
+          <t>Manufacturer code</t>
         </is>
       </c>
     </row>
@@ -12577,6 +12583,11 @@
         <f>IF(OR(W2="",G2=0),"",ROUND(1-W2/G2,3))</f>
         <v/>
       </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>SM58-LCE</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="30">
       <c r="A3" s="48" t="n"/>
@@ -12659,6 +12670,11 @@
         <f>IF(OR(W3="",G3=0),"",ROUND(1-W3/G3,3))</f>
         <v/>
       </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>EW-D 835-S (R1-6)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="30">
       <c r="A4" s="48" t="n"/>
@@ -12740,6 +12756,11 @@
       <c r="X4" s="52">
         <f>IF(OR(W4="",G4=0),"",ROUND(1-W4/G4,3))</f>
         <v/>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>GAF50BK</t>
+        </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="30">
@@ -33746,103 +33767,103 @@
           <t>Sales products: categories</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="29" t="inlineStr">
         <is>
           <t>Sub-Category</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="29" t="inlineStr">
         <is>
           <t>Audio</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="29" t="inlineStr">
         <is>
           <t>General</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="29" t="inlineStr">
         <is>
           <t>Lighting</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="29" t="inlineStr">
         <is>
           <t>General</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="29" t="inlineStr">
         <is>
           <t>Video</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="29" t="inlineStr">
         <is>
           <t>General</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="29" t="inlineStr">
         <is>
           <t>Connectors</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="29" t="inlineStr">
         <is>
           <t>General</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="29" t="inlineStr">
         <is>
           <t>Rigging</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="29" t="inlineStr">
         <is>
           <t>General</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="29" t="inlineStr">
         <is>
           <t>Consumables</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="29" t="inlineStr">
         <is>
           <t>General</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="29" t="inlineStr">
         <is>
           <t>Cases</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="29" t="inlineStr">
         <is>
           <t>General</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" s="29" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="29" t="inlineStr">
         <is>
           <t>General</t>
         </is>

</xml_diff>